<commit_message>
final: the fine-tuned Ornith 9B is the scored solver (r10, pass_rate 0.34)
SOLVER is read from .env.local with ft9b as the default, so judges run their
set against the 9B endpoint without editing code. Root artifacts and the
scores block are the r10 run of the fine-tuned 9B over the 400 tasks.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CatrdSNKb3R1J9vS9deMkH
</commit_message>
<xml_diff>
--- a/outputs/105-24.xlsx
+++ b/outputs/105-24.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="116">
   <si>
     <t xml:space="preserve">Last Extract:</t>
   </si>
@@ -74,6 +74,9 @@
     <t xml:space="preserve">201352340</t>
   </si>
   <si>
+    <t xml:space="preserve">Anuksha Manoj Jaju</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSRL REQ</t>
   </si>
   <si>
@@ -86,9 +89,15 @@
     <t xml:space="preserve">Perform Peer Review</t>
   </si>
   <si>
+    <t xml:space="preserve">Gouthami Jagga</t>
+  </si>
+  <si>
     <t xml:space="preserve">201353834</t>
   </si>
   <si>
+    <t xml:space="preserve">Bekkam Rajashekar</t>
+  </si>
+  <si>
     <t xml:space="preserve">1</t>
   </si>
   <si>
@@ -98,15 +107,27 @@
     <t xml:space="preserve">Awaiting confirmation from site</t>
   </si>
   <si>
+    <t xml:space="preserve">Mahesh Ommi</t>
+  </si>
+  <si>
     <t xml:space="preserve">201354293</t>
   </si>
   <si>
+    <t xml:space="preserve">Chiranjeevi Bollini</t>
+  </si>
+  <si>
     <t xml:space="preserve">Awaiting for Master data confirmation</t>
   </si>
   <si>
+    <t xml:space="preserve">Mamatha Sadineni</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357835</t>
   </si>
   <si>
+    <t xml:space="preserve">Dande Reddy</t>
+  </si>
+  <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
@@ -116,30 +137,48 @@
     <t xml:space="preserve">5 GTIN Setup SLT</t>
   </si>
   <si>
+    <t xml:space="preserve">Manisha Goski</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357814</t>
   </si>
   <si>
+    <t xml:space="preserve">Ramya Kodamanchili</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357820</t>
   </si>
   <si>
     <t xml:space="preserve">21 GTIN setup,see long text</t>
   </si>
   <si>
+    <t xml:space="preserve">Rizwan Ul Hasan Siddiqui</t>
+  </si>
+  <si>
     <t xml:space="preserve">201358099</t>
   </si>
   <si>
     <t xml:space="preserve">Perform peer review</t>
   </si>
   <si>
+    <t xml:space="preserve">Sandeep Kumar</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357884</t>
   </si>
   <si>
     <t xml:space="preserve">1 Partial Batch Decomm, see long text</t>
   </si>
   <si>
+    <t xml:space="preserve">Sravya Reddy</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357586</t>
   </si>
   <si>
+    <t xml:space="preserve">Naraparaju Manasa</t>
+  </si>
+  <si>
     <t xml:space="preserve">8</t>
   </si>
   <si>
@@ -149,9 +188,18 @@
     <t xml:space="preserve">Informed requestor</t>
   </si>
   <si>
+    <t xml:space="preserve">Sriram Podicheti</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357675</t>
   </si>
   <si>
+    <t xml:space="preserve">Rahul Nesarikar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamarala Sisindri</t>
+  </si>
+  <si>
     <t xml:space="preserve">201357932</t>
   </si>
   <si>
@@ -185,6 +233,9 @@
     <t xml:space="preserve">201358396</t>
   </si>
   <si>
+    <t xml:space="preserve">Suneerunnisa Begum</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSOS REQ</t>
   </si>
   <si>
@@ -236,136 +287,85 @@
     <t xml:space="preserve">am427825</t>
   </si>
   <si>
-    <t xml:space="preserve">Anuksha Manoj Jaju</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Russia / Saudi</t>
   </si>
   <si>
     <t xml:space="preserve">br690118</t>
   </si>
   <si>
-    <t xml:space="preserve">Bekkam Rajashekar</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Alerts / US</t>
   </si>
   <si>
     <t xml:space="preserve">cb832551</t>
   </si>
   <si>
-    <t xml:space="preserve">Chiranjeevi Bollini</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Vx</t>
   </si>
   <si>
     <t xml:space="preserve">dvr95541</t>
   </si>
   <si>
-    <t xml:space="preserve">Dande Reddy</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Error Monitoring &amp; Reporting</t>
   </si>
   <si>
     <t xml:space="preserve">gsj65824</t>
   </si>
   <si>
-    <t xml:space="preserve">Gouthami Jagga</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Phase 1</t>
   </si>
   <si>
     <t xml:space="preserve">om209107</t>
   </si>
   <si>
-    <t xml:space="preserve">Mahesh Ommi</t>
-  </si>
-  <si>
     <t xml:space="preserve">ms550164</t>
   </si>
   <si>
-    <t xml:space="preserve">Mamatha Sadineni</t>
-  </si>
-  <si>
     <t xml:space="preserve">Training</t>
   </si>
   <si>
     <t xml:space="preserve">mg104360</t>
   </si>
   <si>
-    <t xml:space="preserve">Manisha Goski</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Phase 2 &amp; ELS Saudi</t>
   </si>
   <si>
     <t xml:space="preserve">nm846496</t>
   </si>
   <si>
-    <t xml:space="preserve">Naraparaju Manasa</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Vx / Error Monitoring &amp; Reporting</t>
   </si>
   <si>
     <t xml:space="preserve">rn545895</t>
   </si>
   <si>
-    <t xml:space="preserve">Rahul Nesarikar</t>
-  </si>
-  <si>
     <t xml:space="preserve">DM / Russia / DV</t>
   </si>
   <si>
     <t xml:space="preserve">rk440576</t>
   </si>
   <si>
-    <t xml:space="preserve">Ramya Kodamanchili</t>
-  </si>
-  <si>
     <t xml:space="preserve">rh294814</t>
   </si>
   <si>
-    <t xml:space="preserve">Rizwan Ul Hasan Siddiqui</t>
-  </si>
-  <si>
     <t xml:space="preserve">spk12633</t>
   </si>
   <si>
-    <t xml:space="preserve">Sandeep Kumar</t>
-  </si>
-  <si>
     <t xml:space="preserve">Alerts / ELS Saudi / Vx</t>
   </si>
   <si>
     <t xml:space="preserve">sr463655</t>
   </si>
   <si>
-    <t xml:space="preserve">Sravya Reddy</t>
-  </si>
-  <si>
     <t xml:space="preserve">sp128618</t>
   </si>
   <si>
-    <t xml:space="preserve">Sriram Podicheti</t>
-  </si>
-  <si>
     <t xml:space="preserve">sb641236</t>
   </si>
   <si>
-    <t xml:space="preserve">Suneerunnisa Begum</t>
-  </si>
-  <si>
     <t xml:space="preserve">Phase 1 / Process Documents</t>
   </si>
   <si>
     <t xml:space="preserve">txs21997</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamarala Sisindri</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -1130,9 +1130,8 @@
       <c r="B4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="11" t="str">
-        <f aca="false">VLOOKUP("am427825",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Anuksha Manoj Jaju</v>
+      <c r="C4" s="11" t="s">
+        <v>17</v>
       </c>
       <c r="D4" s="12" t="n">
         <v>45034</v>
@@ -1142,20 +1141,19 @@
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="11" t="str">
-        <f aca="false">VLOOKUP("gsj65824",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Gouthami Jagga</v>
+        <v>21</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="L4" s="12" t="n">
         <v>45049</v>
@@ -1176,11 +1174,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="11" t="str">
-        <f aca="false">VLOOKUP("br690118",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Bekkam Rajashekar</v>
+        <v>23</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="D5" s="12" t="n">
         <v>45036</v>
@@ -1190,20 +1187,19 @@
       </c>
       <c r="F5" s="11"/>
       <c r="G5" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" s="11" t="str">
-        <f aca="false">VLOOKUP("om209107",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Mahesh Ommi</v>
+        <v>27</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>28</v>
       </c>
       <c r="L5" s="12" t="n">
         <v>45036</v>
@@ -1224,11 +1220,10 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="11" t="str">
-        <f aca="false">VLOOKUP("cb832551",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Chiranjeevi Bollini</v>
+        <v>29</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>45037</v>
@@ -1238,20 +1233,19 @@
       </c>
       <c r="F6" s="11"/>
       <c r="G6" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="K6" s="11" t="str">
-        <f aca="false">VLOOKUP("ms550164",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Mamatha Sadineni</v>
+        <v>31</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="L6" s="12" t="n">
         <v>45037</v>
@@ -1272,11 +1266,10 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="11" t="str">
-        <f aca="false">VLOOKUP("dvr95541",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Dande Reddy</v>
+        <v>33</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>45048</v>
@@ -1286,20 +1279,19 @@
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="11" t="str">
-        <f aca="false">VLOOKUP("mg104360",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Manisha Goski</v>
+        <v>37</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="L7" s="12" t="n">
         <v>45048</v>
@@ -1320,11 +1312,10 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="11" t="str">
-        <f aca="false">VLOOKUP("gsj65824",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Gouthami Jagga</v>
+        <v>39</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>45048</v>
@@ -1334,20 +1325,19 @@
       </c>
       <c r="F8" s="11"/>
       <c r="G8" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="11" t="str">
-        <f aca="false">VLOOKUP("rk440576",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Ramya Kodamanchili</v>
+        <v>21</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="L8" s="12" t="n">
         <v>45050</v>
@@ -1368,11 +1358,10 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="11" t="str">
-        <f aca="false">VLOOKUP("om209107",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Mahesh Ommi</v>
+        <v>41</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>28</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>45049</v>
@@ -1382,20 +1371,19 @@
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" s="11" t="str">
-        <f aca="false">VLOOKUP("rh294814",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rizwan Ul Hasan Siddiqui</v>
+        <v>42</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="L9" s="12" t="n">
         <v>45049</v>
@@ -1416,11 +1404,10 @@
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="11" t="str">
-        <f aca="false">VLOOKUP("ms550164",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Mamatha Sadineni</v>
+        <v>44</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>45049</v>
@@ -1430,20 +1417,19 @@
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="11" t="str">
-        <f aca="false">VLOOKUP("spk12633",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sandeep Kumar</v>
+        <v>45</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>45050</v>
@@ -1464,11 +1450,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="11" t="str">
-        <f aca="false">VLOOKUP("mg104360",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Manisha Goski</v>
+        <v>47</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>45049</v>
@@ -1478,20 +1463,19 @@
       </c>
       <c r="F11" s="11"/>
       <c r="G11" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="K11" s="11" t="str">
-        <f aca="false">VLOOKUP("sr463655",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sravya Reddy</v>
+        <v>48</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>49</v>
       </c>
       <c r="L11" s="12" t="n">
         <v>45050</v>
@@ -1512,11 +1496,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="11" t="str">
-        <f aca="false">VLOOKUP("nm846496",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Naraparaju Manasa</v>
+        <v>50</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>51</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>45048</v>
@@ -1526,20 +1509,19 @@
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="K12" s="11" t="str">
-        <f aca="false">VLOOKUP("sp128618",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sriram Podicheti</v>
+        <v>54</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>55</v>
       </c>
       <c r="L12" s="12" t="n">
         <v>45049</v>
@@ -1560,11 +1542,10 @@
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="11" t="str">
-        <f aca="false">VLOOKUP("rn545895",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rahul Nesarikar</v>
+        <v>56</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>45048</v>
@@ -1574,20 +1555,19 @@
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="K13" s="11" t="str">
-        <f aca="false">VLOOKUP("txs21997",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Tamarala Sisindri</v>
+        <v>54</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>58</v>
       </c>
       <c r="L13" s="12" t="n">
         <v>45050</v>
@@ -1608,11 +1588,10 @@
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="11" t="str">
-        <f aca="false">VLOOKUP("rk440576",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Ramya Kodamanchili</v>
+        <v>59</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>45049</v>
@@ -1622,20 +1601,19 @@
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="K14" s="11" t="str">
-        <f aca="false">VLOOKUP("nm846496",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Naraparaju Manasa</v>
+        <v>54</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>51</v>
       </c>
       <c r="L14" s="12" t="n">
         <v>45050</v>
@@ -1656,11 +1634,10 @@
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="11" t="str">
-        <f aca="false">VLOOKUP("rh294814",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rizwan Ul Hasan Siddiqui</v>
+        <v>60</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>45049</v>
@@ -1670,20 +1647,19 @@
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="K15" s="11" t="str">
-        <f aca="false">VLOOKUP("rn545895",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rahul Nesarikar</v>
+        <v>63</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="L15" s="12" t="n">
         <v>45049</v>
@@ -1704,11 +1680,10 @@
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="11" t="str">
-        <f aca="false">VLOOKUP("spk12633",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sandeep Kumar</v>
+        <v>64</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>45049</v>
@@ -1718,20 +1693,19 @@
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="K16" s="11" t="str">
-        <f aca="false">VLOOKUP("spk12633",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sandeep Kumar</v>
+        <v>48</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="L16" s="12" t="n">
         <v>45050</v>
@@ -1752,11 +1726,10 @@
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>49</v>
-      </c>
-      <c r="C17" s="11" t="str">
-        <f aca="false">VLOOKUP("sr463655",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sravya Reddy</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>45050</v>
@@ -1766,20 +1739,19 @@
       </c>
       <c r="F17" s="11"/>
       <c r="G17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="K17" s="11" t="s">
         <v>17</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="K17" s="11" t="str">
-        <f aca="false">VLOOKUP("am427825",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Anuksha Manoj Jaju</v>
       </c>
       <c r="L17" s="12" t="n">
         <v>45050</v>
@@ -1800,11 +1772,10 @@
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="11" t="str">
-        <f aca="false">VLOOKUP("sp128618",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sriram Podicheti</v>
+        <v>67</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>55</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>45050</v>
@@ -1814,20 +1785,19 @@
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="K18" s="11" t="str">
-        <f aca="false">VLOOKUP("br690118",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Bekkam Rajashekar</v>
+        <v>68</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="L18" s="12" t="n">
         <v>45050</v>
@@ -1848,11 +1818,10 @@
     </row>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="11" t="str">
-        <f aca="false">VLOOKUP("sb641236",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Suneerunnisa Begum</v>
+        <v>69</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>70</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>45050</v>
@@ -1862,20 +1831,19 @@
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="K19" s="11" t="str">
-        <f aca="false">VLOOKUP("cb832551",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Chiranjeevi Bollini</v>
+        <v>72</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="L19" s="12" t="n">
         <v>45050</v>
@@ -1894,11 +1862,10 @@
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="11" t="str">
-        <f aca="false">VLOOKUP("txs21997",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Tamarala Sisindri</v>
+        <v>73</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>58</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>45050</v>
@@ -1908,20 +1875,19 @@
       </c>
       <c r="F20" s="11"/>
       <c r="G20" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="K20" s="11" t="str">
-        <f aca="false">VLOOKUP("dvr95541",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Dande Reddy</v>
+        <v>74</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="L20" s="12" t="n">
         <v>45050</v>
@@ -1942,11 +1908,10 @@
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" s="11" t="str">
-        <f aca="false">VLOOKUP("nm846496",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Naraparaju Manasa</v>
+        <v>75</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>51</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>45050</v>
@@ -1956,20 +1921,19 @@
       </c>
       <c r="F21" s="11"/>
       <c r="G21" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="K21" s="11" t="str">
-        <f aca="false">VLOOKUP("rh294814",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rizwan Ul Hasan Siddiqui</v>
+        <v>21</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="L21" s="12" t="n">
         <v>45050</v>
@@ -1990,11 +1954,10 @@
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="11" t="str">
-        <f aca="false">VLOOKUP("rn545895",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Rahul Nesarikar</v>
+        <v>76</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>44980</v>
@@ -2004,20 +1967,19 @@
       </c>
       <c r="F22" s="11"/>
       <c r="G22" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="K22" s="11" t="str">
-        <f aca="false">VLOOKUP("spk12633",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sandeep Kumar</v>
+        <v>77</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="L22" s="12" t="n">
         <v>44980</v>
@@ -2038,11 +2000,10 @@
     </row>
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="11" t="str">
-        <f aca="false">VLOOKUP("spk12633",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sandeep Kumar</v>
+        <v>78</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>45049</v>
@@ -2052,20 +2013,19 @@
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="K23" s="11" t="str">
-        <f aca="false">VLOOKUP("sr463655",Productivity!$A$4:$B$20,2,FALSE())</f>
-        <v>Sravya Reddy</v>
+        <v>63</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>49</v>
       </c>
       <c r="L23" s="12" t="n">
         <v>45049</v>
@@ -2114,12 +2074,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
       <c r="D1" s="15" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E1" s="15"/>
     </row>
@@ -2128,244 +2088,244 @@
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
       <c r="D2" s="16" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="E2" s="16"/>
     </row>
     <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D4" s="22"/>
       <c r="E4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D5" s="22"/>
       <c r="E5" s="22"/>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D9" s="22"/>
       <c r="E9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>91</v>
+        <v>38</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>97</v>
+        <v>57</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>99</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>89</v>
       </c>
       <c r="D14" s="22"/>
       <c r="E14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D15" s="22"/>
       <c r="E15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>104</v>
+        <v>46</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D16" s="22"/>
       <c r="E16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>109</v>
+        <v>55</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>

</xml_diff>